<commit_message>
Excel templates and import rows for six more lists; Corporal Location and Systemic Therapy aligned with the step-1 workbook; import script treats more 'nothing new' messages as present
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HPB_Templates/Corporal Location_export.xlsx
+++ b/HPB_Templates/Corporal Location_export.xlsx
@@ -530,6 +530,96 @@
       </c>
       <c r="C14" s="3" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1">
+        <v>14.0</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Pancreas primary</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Primary tumour in the pancreas (site not further specified); diagnostic specimen site in the step-1 data sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1">
+        <v>15.0</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Liver metastasis</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Metastasis in the liver; diagnostic specimen site in the step-1 data sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1">
+        <v>16.0</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Peritoneum</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Peritoneal disease or peritoneal specimen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Node</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Lymph node</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Effusion</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Pleural or ascitic effusion (cytology)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1">
+        <v>19.0</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Other specimen site</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>